<commit_message>
Updated - HSCODE - REMOVE ADD AND EDIT AND DELETE - st.run
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -716,7 +716,11 @@
           <t>94038, 94033, 94035, 94036</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated - HSCODE - Add - Edit
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B47A813-8F59-4404-8653-5076B1ABD6A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE043976-51FA-4FF7-8106-B1979E4164C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="750" windowWidth="29040" windowHeight="15570" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="750" windowWidth="29040" windowHeight="15570" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="YANWEN NOVA PGA HS CODE" sheetId="1" r:id="rId1"/>

</xml_diff>